<commit_message>
wip: blog module progress - create, verify, approve, unpublish flow
</commit_message>
<xml_diff>
--- a/resources/UserDetails_beta.xlsx
+++ b/resources/UserDetails_beta.xlsx
@@ -528,7 +528,7 @@
     </border>
   </borders>
   <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1217,47 +1217,47 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <sheetData>
     <row r="1" spans="1:1">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="s" s="0">
+    <row r="2" spans="1:1">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="s" s="0">
+    <row r="3" spans="1:1">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
+    <row r="4" spans="1:1">
+      <c r="A4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="s" s="0">
+    <row r="5" spans="1:1">
+      <c r="A5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="s" s="0">
+    <row r="6" spans="1:1">
+      <c r="A6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="s" s="0">
+    <row r="7" spans="1:1">
+      <c r="A7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="s" s="0">
+    <row r="8" spans="1:1">
+      <c r="A8" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="s" s="0">
+    <row r="9" spans="1:1">
+      <c r="A9" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>